<commit_message>
Package 0.3.1: follow the external clock rate (driver 0.2.2, panel 1.5)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project/PROVENANCE-MATRIX-AUDIOPHILE.xlsx
+++ b/docs/project/PROVENANCE-MATRIX-AUDIOPHILE.xlsx
@@ -1017,7 +1017,7 @@
     <row r="2">
       <c r="A2" s="78" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -1056,7 +1056,7 @@
       </c>
       <c r="D6" s="70" t="inlineStr">
         <is>
-          <t>Pacote 0.2.2 (driver 0.2.0, painel 1.3) publicado (v0.2.2, R122) e instalado no MacBook Air por atualização. Usuário (R123): tudo funcionando; S/PDIF do POD X3 trava em todas as taxas (taxa ajustada à mão); desinstalador e menu de status funcionam.</t>
+          <t>Pacote 0.2.2 (driver 0.2.0, painel 1.3) publicado (v0.2.2, R122). Pacote 0.3.1 (driver 0.2.2, painel 1.5; Classic + Modern) é build de teste, não publicado: seguir a taxa do relógio externo (AP-5.7) funciona no Modern com o FW1814 e o POD X3 (captura 99, R131).</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="D11" s="70" t="inlineStr">
         <is>
-          <t>Sem testes formais (R123): os testes restantes estão como 'Sob demanda (uso real)' e só voltam se o uso real mostrar problema. Próximo trabalho só por pedido do usuário (limpeza de diagnósticos, novos modelos).</t>
+          <t>Sem testes formais (R123). Próximo, só por pedido: gerar o Classic 0.3.1 e os .dmg, commit, publicar 0.3.x (README: edições + seguir a taxa externa) com o OK do usuário; depois limpeza de diagnósticos, novos modelos.</t>
         </is>
       </c>
     </row>
@@ -7155,7 +7155,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I66"/>
+  <dimension ref="A1:I67"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" style="21" min="1" max="1"/>
@@ -10224,7 +10224,7 @@
         </is>
       </c>
     </row>
-    <row r="66">
+    <row r="66" s="21">
       <c r="A66" s="95" t="inlineStr">
         <is>
           <t>AP-5.6</t>
@@ -10268,6 +10268,53 @@
       <c r="I66" s="51" t="inlineStr">
         <is>
           <t>[2026-10-21] Código no commit e9341bb; make test do painel ALL PASS no iMac. R118. Falta ver ao vivo com música. [2026-10-21] R118 registrado. [2026-10-21] Medidor grande em uso no Air (R122, CPU medida); usuário: tudo funcionando (R123).</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" s="21">
+      <c r="A67" s="95" t="inlineStr">
+        <is>
+          <t>AP-5.7</t>
+        </is>
+      </c>
+      <c r="B67" s="96" t="inlineStr">
+        <is>
+          <t>5</t>
+        </is>
+      </c>
+      <c r="C67" s="96" t="inlineStr">
+        <is>
+          <t>Seguir a taxa do relógio externo (kext publica MAExternalSyncRate; painel segue pela CoreAudio)</t>
+        </is>
+      </c>
+      <c r="D67" s="96" t="inlineStr">
+        <is>
+          <t>Testes host do RateFollower; no hardware (1814 + POD X3, nosso driver): 44.1/48/88.2/96 a partir de 48 e de 96, ocioso e com cliente tocando</t>
+        </is>
+      </c>
+      <c r="E67" s="96" t="inlineStr">
+        <is>
+          <t>AP-5.5</t>
+        </is>
+      </c>
+      <c r="F67" s="96" t="inlineStr">
+        <is>
+          <t>Concluído</t>
+        </is>
+      </c>
+      <c r="G67" s="96" t="inlineStr">
+        <is>
+          <t>Claude + Você</t>
+        </is>
+      </c>
+      <c r="H67" s="96" t="inlineStr">
+        <is>
+          <t>RATE_FOLLOW_PLAN_v1</t>
+        </is>
+      </c>
+      <c r="I67" s="51" t="inlineStr">
+        <is>
+          <t>[2026-10-22] Captura 98 no rig SL (driver oficial 1.9, POD X3 por S/PDIF coaxial): o 1814 informa a taxa exata da fonte dentro da faixa de velocidade atual (44.1/48 ou 88.2/96), nada fora dela; o driver oficial publica MASampleRate mas não segue. Decisões do usuário: só ocioso, opção ligada por padrão, uma tentativa da outra faixa. Código: kext (FWAudioDeviceProps.cpp DetectExternalSyncChanges), painel (RateFollower.swift, aba Hardware, menu de status). Kext Classic (build PC) e Modern (Mac dev) compilam; make test do painel ALL PASS e typecheck limpo no iMac. Falta: pacote e teste no hardware com o usuário. R131. [2026-10-22] Pacote 0.3.1 Modern (driver 0.2.2, painel 1.5) instalado pelo usuário no Mac dev (14.8.9) com o segundo FW1814 (0xD6C040074B9FB) e o POD X3: fora da faixa troca a faixa de velocidade, dentro da faixa pega a taxa exata e trava. Usuário: 'worked PERFECT'. Captura 99, R131. Classic 0.3.1 ainda não gerado.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
0.4.0: FireWire 410 support (driver 0.3.0, panel 1.6), stereo pairs as CoreAudio devices, unload / power-off panic fixes; README for three interfaces
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/project/PROVENANCE-MATRIX-AUDIOPHILE.xlsx
+++ b/docs/project/PROVENANCE-MATRIX-AUDIOPHILE.xlsx
@@ -1056,7 +1056,7 @@
       </c>
       <c r="D6" s="70" t="inlineStr">
         <is>
-          <t>Pacote 0.2.2 (driver 0.2.0, painel 1.3) publicado (v0.2.2, R122). Pacote 0.3.1 (driver 0.2.2, painel 1.5; Classic + Modern) é build de teste, não publicado: seguir a taxa do relógio externo (AP-5.7) funciona no Modern com o FW1814 e o POD X3 (captura 99, R131).</t>
+          <t>Pacote 0.3.1 (driver 0.2.2, painel 1.5; Classic + Modern) publicado (v0.3.1). Pânico ao acordar do sleep no Modern com o FW1814 (R133): corrigido no código, driver 0.2.3; pacote 0.3.2 Modern (teste, não publicado) construído, aguarda instalação no dev Mac.</t>
         </is>
       </c>
     </row>
@@ -1121,7 +1121,7 @@
       </c>
       <c r="D11" s="70" t="inlineStr">
         <is>
-          <t>Sem testes formais (R123). Próximo, só por pedido: gerar o Classic 0.3.1 e os .dmg, commit, publicar 0.3.x (README: edições + seguir a taxa externa) com o OK do usuário; depois limpeza de diagnósticos, novos modelos.</t>
+          <t>Sem testes formais (R123). Próximo: o usuário instala o 0.3.2 Modern e usa com sleep/wake. Só por pedido: Classic 0.3.2 e os .dmg, commit, publicar v0.3.2 (gh release); depois limpeza de diagnósticos, novos modelos.</t>
         </is>
       </c>
     </row>
@@ -8654,7 +8654,7 @@
       </c>
       <c r="F32" s="96" t="inlineStr">
         <is>
-          <t>Sob demanda (uso real)</t>
+          <t>Aguarda o usuário</t>
         </is>
       </c>
       <c r="G32" s="96" t="inlineStr">
@@ -8669,7 +8669,7 @@
       </c>
       <c r="I32" s="96" t="inlineStr">
         <is>
-          <t>[2026-10-20] Código pronto: fila AV/C assíncrona segura no teardown (referência na unidade por comando, drenagem + cancel no stop), anel de diagnóstico com lock e traços Rev2. Critério kextunload x5 na fase 7. R107. [2026-10-20] [2026-10-20] captura 97, R117: correção do vazamento de host plug (FreeHostPlugs); unload x5 não executado (decisão do usuário: instalador não descarrega). [2026-10-21] Anel e teardown prontos (R107, R117); kextunload x5 não feito (instalador nunca descarrega). Política R123 (usuário): sem testes formais; só se o uso real mostrar problema.</t>
+          <t>[2026-10-20] Código pronto: fila AV/C assíncrona segura no teardown (referência na unidade por comando, drenagem + cancel no stop), anel de diagnóstico com lock e traços Rev2. Critério kextunload x5 na fase 7. R107. [2026-10-20] [2026-10-20] captura 97, R117: correção do vazamento de host plug (FreeHostPlugs); unload x5 não executado (decisão do usuário: instalador não descarrega). [2026-10-21] Anel e teardown prontos (R107, R117); kextunload x5 não feito (instalador nunca descarrega). Política R123 (usuário): sem testes formais; só se o uso real mostrar problema. [2026-10-22] R133: pânico ao acordar do sleep no dev Mac (Modern 0.3.1, FW1814 0xD6C040074B9FB): StartQueueHead liberava duas vezes um comando AV/C recusado na hora (o callback já o tinha finalizado dentro do submit, IOFireWireAVC-436 :305-306). Correção: retain durante o submit + checagem de head; driver 0.2.3, pacote 0.3.2 Modern construído (kext 4EB8D407). Aguarda instalação pelo usuário e uso real com sleep/wake.</t>
         </is>
       </c>
     </row>
@@ -9515,7 +9515,7 @@
       </c>
       <c r="I50" s="96" t="inlineStr">
         <is>
-          <t>[2026-10-20] [2026-10-20] captura 97, R117: power-cycle das duas unidades com o driver carregado ok; soak 30 s das duas juntas ok; sleep/wake, MIDI, soak 1 h pendentes. [2026-10-21] Power-cycle ok (R117). Soak dispensado (usuário: inútil). Sleep/wake e MIDI no fio: Política R123 (usuário): sem testes formais; só se o uso real mostrar problema.</t>
+          <t>[2026-10-20] [2026-10-20] captura 97, R117: power-cycle das duas unidades com o driver carregado ok; soak 30 s das duas juntas ok; sleep/wake, MIDI, soak 1 h pendentes. [2026-10-21] Power-cycle ok (R117). Soak dispensado (usuário: inútil). Sleep/wake e MIDI no fio: Política R123 (usuário): sem testes formais; só se o uso real mostrar problema. [2026-10-22] Sleep/wake: uso real mostrou pânico ao acordar (R133), corrigido no código (driver 0.2.3); verificação = uso real após instalar 0.3.2.</t>
         </is>
       </c>
     </row>

</xml_diff>